<commit_message>
ADMM models. Update to consider vmag_sqr, pc_node, qc_node.
</commit_message>
<xml_diff>
--- a/data/CS7/Market Data/CS7_market_data_2025.xlsx
+++ b/data/CS7/Market Data/CS7_market_data_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\thesis-shared-resources-planning-no_esso-degradation\data\CS7\Market Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B2F5F9A-BC28-45FD-865A-6613F49C44FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D9955A-A76F-4C1A-9918-0D00908AF1CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-15195" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2237,19 +2237,19 @@
         <v>1</v>
       </c>
       <c r="B1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1">
         <f>1/$B$1</f>
-        <v>1</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D1" s="1">
         <f t="shared" ref="D1:E1" si="0">1/$B$1</f>
-        <v>1</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E1" s="1">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>

</xml_diff>

<commit_message>
Network model. Shared ESS. Simplified extended formulation added.
</commit_message>
<xml_diff>
--- a/data/CS7/Market Data/CS7_market_data_2025.xlsx
+++ b/data/CS7/Market Data/CS7_market_data_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\thesis-shared-resources-planning-no_esso-degradation\data\CS7\Market Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D9955A-A76F-4C1A-9918-0D00908AF1CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84454AF3-C07D-4657-843A-E8DF1F6BFACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-15195" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33120" yWindow="-10755" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="1" r:id="rId1"/>

</xml_diff>